<commit_message>
tabtools: add SSC release plan, gate tests, and QA updates
</commit_message>
<xml_diff>
--- a/tabtools/qa/output_issue_rendering/crosstab_boldp.xlsx
+++ b/tabtools/qa/output_issue_rendering/crosstab_boldp.xlsx
@@ -61,7 +61,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="208">
+  <fonts count="218">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -631,6 +631,46 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -935,7 +975,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="152">
+  <borders count="162">
     <border>
       <left/>
       <right/>
@@ -1856,105 +1896,175 @@
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
+      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
@@ -1968,7 +2078,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -2491,71 +2601,111 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="183" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="184" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="185" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="186" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="187" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="189" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="191" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="193" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="195" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="197" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="199" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="201" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="203" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="205" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="207" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="146" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="147" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="148" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="149" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="150" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="151" xfId="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="188" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="189" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="190" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="191" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="192" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="193" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="194" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="195" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="196" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="197" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="199" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="201" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="203" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="205" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="207" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="209" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="211" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="213" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="215" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="217" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="156" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="157" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="158" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="159" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="160" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="161" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2568,12 +2718,12 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="146" customWidth="true"/>
-    <col min="2" max="2" width="12.7109375" style="147" customWidth="true"/>
-    <col min="3" max="3" width="14.7109375" style="148" customWidth="true"/>
-    <col min="4" max="4" width="14.7109375" style="149" customWidth="true"/>
-    <col min="5" max="5" width="14.7109375" style="150" customWidth="true"/>
-    <col min="6" max="6" width="14.7109375" style="151" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="156" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" style="157" customWidth="true"/>
+    <col min="3" max="3" width="14.7109375" style="158" customWidth="true"/>
+    <col min="4" max="4" width="14.7109375" style="159" customWidth="true"/>
+    <col min="5" max="5" width="14.7109375" style="160" customWidth="true"/>
+    <col min="6" max="6" width="14.7109375" style="161" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2680,19 +2830,19 @@
       <c r="A6" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="136" t="s">
+      <c r="B6" s="146" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="137" t="s">
+      <c r="C6" s="147" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="138" t="s">
+      <c r="D6" s="148" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="139" t="s">
+      <c r="E6" s="149" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="140" t="s">
+      <c r="F6" s="150" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2700,25 +2850,26 @@
       <c r="A7" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="141" t="s">
+      <c r="B7" s="151" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="142" t="s">
+      <c r="C7" s="152" t="s">
         <v>0</v>
       </c>
-      <c r="D7" s="143" t="s">
+      <c r="D7" s="153" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="144" t="s">
+      <c r="E7" s="154" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="145" t="s">
+      <c r="F7" s="155" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B7:F7"/>
   </mergeCells>
 </worksheet>

</xml_diff>